<commit_message>
Update LeaveApproved: add request date column & add show file, WorkLog: show gps
</commit_message>
<xml_diff>
--- a/WebContent/upload/template/report_leaveapprove.xlsx
+++ b/WebContent/upload/template/report_leaveapprove.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="27307"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10531"/>
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\CubeSoft\CA\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juneog/eclipse-workspace/cube/CA-II/WebContent/upload/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{38A63D6F-B761-485C-92F1-EA36B538753D}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295F7E7F-9982-024C-BFD8-260C07D04149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="12456" xr2:uid="{FA967C5A-5BC9-4416-8971-A23587205F3B}"/>
+    <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" xr2:uid="{FA967C5A-5BC9-4416-8971-A23587205F3B}"/>
   </bookViews>
   <sheets>
     <sheet name="Report" sheetId="1" r:id="rId1"/>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
   <si>
     <t>รายงานการลางานของพนักงาน</t>
   </si>
@@ -91,6 +91,9 @@
   </si>
   <si>
     <t>Status</t>
+  </si>
+  <si>
+    <t>Request Date</t>
   </si>
 </sst>
 </file>
@@ -104,7 +107,7 @@
     <font>
       <sz val="11"/>
       <color theme="1"/>
-      <name val="Calibri"/>
+      <name val="Tahoma"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
@@ -164,7 +167,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="6">
+  <borders count="5">
     <border>
       <left/>
       <right/>
@@ -230,24 +233,11 @@
       </bottom>
       <diagonal/>
     </border>
-    <border>
-      <left/>
-      <right style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </right>
-      <top style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </top>
-      <bottom style="thin">
-        <color theme="0" tint="-0.14999847407452621"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="27">
+  <cellXfs count="24">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
@@ -279,30 +269,25 @@
     <xf numFmtId="0" fontId="6" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1"/>
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment horizontal="center"/>
     </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="4" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="3" borderId="5" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="6" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="7" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="ปกติ" xfId="0" builtinId="0"/>
@@ -390,9 +375,9 @@
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
-<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="Office Theme">
+<a:theme xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" name="ธีม Office 2013 - 2022">
   <a:themeElements>
-    <a:clrScheme name="Office">
+    <a:clrScheme name="Office 2013 - 2022">
       <a:dk1>
         <a:sysClr val="windowText" lastClr="000000"/>
       </a:dk1>
@@ -430,7 +415,7 @@
         <a:srgbClr val="954F72"/>
       </a:folHlink>
     </a:clrScheme>
-    <a:fontScheme name="Office">
+    <a:fontScheme name="Office 2013 - 2022">
       <a:majorFont>
         <a:latin typeface="Calibri Light" panose="020F0302020204030204"/>
         <a:ea typeface=""/>
@@ -536,7 +521,7 @@
         <a:font script="Tfng" typeface="Ebrima"/>
       </a:minorFont>
     </a:fontScheme>
-    <a:fmtScheme name="Office">
+    <a:fmtScheme name="Office 2013 - 2022">
       <a:fillStyleLst>
         <a:solidFill>
           <a:schemeClr val="phClr"/>
@@ -678,7 +663,7 @@
   <a:extraClrSchemeLst/>
   <a:extLst>
     <a:ext uri="{05A4C25C-085E-4340-85A3-A5531E510DB2}">
-      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
+      <thm15:themeFamily xmlns:thm15="http://schemas.microsoft.com/office/thememl/2012/main" name="Office 2013 - 2022 Theme" id="{62F939B6-93AF-4DB8-9C6B-D6C7DFDC589F}" vid="{4A3C46E8-61CC-4603-A589-7422A47A8E4A}"/>
     </a:ext>
   </a:extLst>
 </a:theme>
@@ -687,23 +672,23 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{705E816A-1600-4C6E-B044-313BAADE2790}">
   <dimension ref="A1:X6"/>
-  <sheetFormatPr defaultColWidth="18.7109375" defaultRowHeight="16.149999999999999" customHeight="1"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="18.6640625" defaultRowHeight="16.25" customHeight="1"/>
   <cols>
-    <col min="1" max="1" width="18.7109375" style="3"/>
-    <col min="2" max="2" width="48.28515625" style="3" customWidth="1"/>
-    <col min="3" max="3" width="28.85546875" style="3" customWidth="1"/>
-    <col min="4" max="4" width="26.28515625" style="3" customWidth="1"/>
-    <col min="5" max="5" width="25.7109375" style="3" customWidth="1"/>
-    <col min="6" max="6" width="30.7109375" style="3" customWidth="1"/>
-    <col min="7" max="12" width="33.42578125" style="3" customWidth="1"/>
-    <col min="13" max="16384" width="18.7109375" style="3"/>
+    <col min="1" max="1" width="18.6640625" style="3"/>
+    <col min="2" max="2" width="48.33203125" style="3" customWidth="1"/>
+    <col min="3" max="3" width="28.83203125" style="3" customWidth="1"/>
+    <col min="4" max="4" width="26.33203125" style="3" customWidth="1"/>
+    <col min="5" max="5" width="25.6640625" style="3" customWidth="1"/>
+    <col min="6" max="6" width="30.6640625" style="3" customWidth="1"/>
+    <col min="7" max="12" width="33.5" style="3" customWidth="1"/>
+    <col min="13" max="16384" width="18.6640625" style="3"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:24" ht="72" customHeight="1">
-      <c r="A1" s="15" t="e" vm="1">
+      <c r="A1" s="22" t="e" vm="1">
         <v>#VALUE!</v>
       </c>
-      <c r="B1" s="15"/>
+      <c r="B1" s="22"/>
       <c r="C1" s="1" t="s">
         <v>0</v>
       </c>
@@ -711,14 +696,14 @@
       <c r="E1" s="2"/>
       <c r="F1" s="2"/>
     </row>
-    <row r="2" spans="1:24" ht="16.149999999999999" customHeight="1">
-      <c r="A2" s="17"/>
-      <c r="B2" s="18"/>
-      <c r="C2" s="18"/>
-      <c r="D2" s="18"/>
-      <c r="E2" s="18"/>
+    <row r="2" spans="1:24" ht="16.25" customHeight="1">
+      <c r="A2" s="23"/>
+      <c r="B2" s="21"/>
+      <c r="C2" s="21"/>
+      <c r="D2" s="21"/>
+      <c r="E2" s="21"/>
     </row>
-    <row r="3" spans="1:24" s="8" customFormat="1" ht="16.149999999999999" customHeight="1">
+    <row r="3" spans="1:24" s="8" customFormat="1" ht="16.25" customHeight="1">
       <c r="A3" s="8" t="s">
         <v>1</v>
       </c>
@@ -728,27 +713,24 @@
       </c>
       <c r="E3" s="10"/>
       <c r="G3" s="11"/>
-      <c r="L3" s="25"/>
-      <c r="M3" s="26"/>
-      <c r="N3" s="26"/>
-      <c r="O3" s="26"/>
+      <c r="L3" s="19"/>
+      <c r="M3" s="20"/>
+      <c r="N3" s="20"/>
+      <c r="O3" s="20"/>
     </row>
-    <row r="4" spans="1:24" ht="16.149999999999999" customHeight="1">
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="18"/>
-      <c r="E4" s="18"/>
-      <c r="G4" s="19"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
+    <row r="4" spans="1:24" ht="16.25" customHeight="1">
+      <c r="B4" s="23"/>
+      <c r="C4" s="21"/>
+      <c r="D4" s="21"/>
+      <c r="E4" s="21"/>
+      <c r="G4" s="4"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
     </row>
-    <row r="5" spans="1:24" s="7" customFormat="1" ht="49.9" customHeight="1">
+    <row r="5" spans="1:24" s="7" customFormat="1" ht="50" customHeight="1">
       <c r="A5" s="13" t="s">
         <v>3</v>
       </c>
@@ -767,16 +749,18 @@
       <c r="F5" s="14" t="s">
         <v>8</v>
       </c>
-      <c r="G5" s="16" t="s">
+      <c r="G5" s="15" t="s">
         <v>9</v>
       </c>
-      <c r="H5" s="24" t="s">
+      <c r="H5" s="18" t="s">
         <v>10</v>
       </c>
-      <c r="I5" s="23"/>
-      <c r="J5" s="21"/>
-      <c r="K5" s="21"/>
-      <c r="L5" s="22"/>
+      <c r="I5" s="18" t="s">
+        <v>11</v>
+      </c>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="17"/>
       <c r="M5" s="12"/>
       <c r="N5" s="12"/>
       <c r="O5" s="12"/>
@@ -790,7 +774,7 @@
       <c r="W5" s="12"/>
       <c r="X5" s="12"/>
     </row>
-    <row r="6" spans="1:24" ht="13.9">
+    <row r="6" spans="1:24" ht="17">
       <c r="A6" s="4"/>
       <c r="B6" s="4"/>
       <c r="C6" s="4"/>

</xml_diff>

<commit_message>
Update Leave Approved : add remark column for export excel
</commit_message>
<xml_diff>
--- a/WebContent/upload/template/report_leaveapprove.xlsx
+++ b/WebContent/upload/template/report_leaveapprove.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/juneog/eclipse-workspace/cube/CA-II/WebContent/upload/template/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{295F7E7F-9982-024C-BFD8-260C07D04149}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{66C52C6D-0BB3-8243-B24F-C31167EC15E9}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="0" yWindow="600" windowWidth="23260" windowHeight="12460" xr2:uid="{FA967C5A-5BC9-4416-8971-A23587205F3B}"/>
   </bookViews>
@@ -58,7 +58,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="12" uniqueCount="12">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="13" uniqueCount="13">
   <si>
     <t>รายงานการลางานของพนักงาน</t>
   </si>
@@ -94,6 +94,9 @@
   </si>
   <si>
     <t>Request Date</t>
+  </si>
+  <si>
+    <t>Remark</t>
   </si>
 </sst>
 </file>
@@ -758,7 +761,9 @@
       <c r="I5" s="18" t="s">
         <v>11</v>
       </c>
-      <c r="J5" s="16"/>
+      <c r="J5" s="18" t="s">
+        <v>12</v>
+      </c>
       <c r="K5" s="16"/>
       <c r="L5" s="17"/>
       <c r="M5" s="12"/>

</xml_diff>